<commit_message>
j'essaie de créer un dictionnaire député>groupe>couleur pour coloier les points mais ligne 205 je ne trouve pas de correspondance en utilisant DEPUTES_FILE
</commit_message>
<xml_diff>
--- a/Graphe.xlsx
+++ b/Graphe.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thomas.platz\PycharmProjects\Deputes2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E1F440B8-BE7D-4F89-B729-32E88ADAFDA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{790FE19F-41B7-4520-B156-915DFF2EDD4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1D6707C7-54AC-49DF-A0B7-A74DEF07AF2F}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="34">
   <si>
     <t>v1</t>
   </si>
@@ -143,13 +143,16 @@
     <t>7.161413</t>
   </si>
   <si>
-    <t>Column1</t>
+    <t>x</t>
   </si>
   <si>
-    <t>Column2</t>
+    <t>y</t>
   </si>
   <si>
-    <t>Column3</t>
+    <t>label</t>
+  </si>
+  <si>
+    <t>l</t>
   </si>
 </sst>
 </file>
@@ -165,15 +168,21 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -181,18 +190,64 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -229,58 +284,65 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:chart>
-    <c:title>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="fr-FR"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
+    <c:autoTitleDeleted val="1"/>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="6.0644552536734952E-2"/>
+          <c:y val="5.9846108570977392E-2"/>
+          <c:w val="0.92345082703588222"/>
+          <c:h val="0.80420075539338065"/>
+        </c:manualLayout>
+      </c:layout>
       <c:scatterChart>
         <c:scatterStyle val="lineMarker"/>
         <c:varyColors val="0"/>
         <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
+          <c:idx val="1"/>
+          <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>'coordinates'!$C$1</c:f>
+              <c:f>'coordinates'!$A$2:$A$11</c:f>
               <c:strCache>
-                <c:ptCount val="1"/>
+                <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>Column3</c:v>
+                  <c:v>v1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>v2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>v3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>v4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>v5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>v6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>v7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>v8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>v9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>v10</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:ln w="38100" cap="rnd">
+            <a:ln w="25400" cap="rnd">
               <a:noFill/>
               <a:round/>
             </a:ln>
@@ -291,54 +353,486 @@
             <c:size val="5"/>
             <c:spPr>
               <a:solidFill>
-                <a:schemeClr val="accent1"/>
+                <a:schemeClr val="accent2"/>
               </a:solidFill>
               <a:ln w="9525">
                 <a:solidFill>
-                  <a:schemeClr val="accent1"/>
+                  <a:schemeClr val="accent2"/>
                 </a:solidFill>
               </a:ln>
               <a:effectLst/>
             </c:spPr>
           </c:marker>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="0"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{7EEA96EE-1E96-4142-882B-67FD66FB23F6}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[PLAGECELL]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="fr-FR"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000003-F99D-46D1-A11D-727F70D9B603}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{57307F41-8809-4458-B170-5759B2117FCB}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[PLAGECELL]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="fr-FR"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000004-F99D-46D1-A11D-727F70D9B603}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="2"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{E0C7BD9F-61EB-450E-A8A0-2C67C4F6CF5A}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[PLAGECELL]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="fr-FR"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000005-F99D-46D1-A11D-727F70D9B603}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="3"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{B9305632-3594-4FFD-B8B2-2DC18017DB97}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[PLAGECELL]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="fr-FR"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000006-F99D-46D1-A11D-727F70D9B603}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="4"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{1101877C-7A7D-47E5-BBC9-710274F168C2}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[PLAGECELL]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="fr-FR"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000007-F99D-46D1-A11D-727F70D9B603}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="5"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{FD9470B4-549A-459B-88FF-5F1D6B776BB8}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[PLAGECELL]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="fr-FR"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000008-F99D-46D1-A11D-727F70D9B603}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="6"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{3907B7CC-60AD-4D70-8986-184883EFB80F}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[PLAGECELL]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="fr-FR"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000009-F99D-46D1-A11D-727F70D9B603}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="7"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{BDDF63A6-BF2A-4B24-9118-1C2F2145533E}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[PLAGECELL]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="fr-FR"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{0000000A-F99D-46D1-A11D-727F70D9B603}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="8"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{E397FBF1-784B-4AFD-9EB7-6A2AC94CB666}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[PLAGECELL]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="fr-FR"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{0000000B-F99D-46D1-A11D-727F70D9B603}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="9"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{AAEDB36A-EC71-4B15-B366-B547848DAB6A}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[PLAGECELL]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="fr-FR"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{0000000C-F99D-46D1-A11D-727F70D9B603}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="fr-FR"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="t"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showDataLabelsRange val="1"/>
+                <c15:showLeaderLines val="0"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:xVal>
-            <c:multiLvlStrRef>
-              <c:f>'coordinates'!$A$2:$B$11</c:f>
-              <c:multiLvlStrCache>
+            <c:numRef>
+              <c:f>'coordinates'!$B$2:$B$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
-                <c:lvl>
-                  <c:pt idx="0">
-                    <c:v>-8.992044</c:v>
-                  </c:pt>
-                  <c:pt idx="1">
-                    <c:v>-8.974819</c:v>
-                  </c:pt>
-                  <c:pt idx="2">
-                    <c:v>-8.446354</c:v>
-                  </c:pt>
-                  <c:pt idx="3">
-                    <c:v>-11.709638</c:v>
-                  </c:pt>
-                  <c:pt idx="4">
-                    <c:v>-12.038005</c:v>
-                  </c:pt>
-                  <c:pt idx="5">
-                    <c:v>-12.226768</c:v>
-                  </c:pt>
-                  <c:pt idx="6">
-                    <c:v>-11.559609</c:v>
-                  </c:pt>
-                  <c:pt idx="7">
-                    <c:v>-11.7438965</c:v>
-                  </c:pt>
-                  <c:pt idx="8">
-                    <c:v>-12.1509905</c:v>
-                  </c:pt>
-                  <c:pt idx="9">
-                    <c:v>-11.58899</c:v>
-                  </c:pt>
-                </c:lvl>
-                <c:lvl>
+                <c:pt idx="0">
+                  <c:v>-8.9920439999999999</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-8.9748190000000001</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-8.4463539999999995</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-11.709638</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-12.038005</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-12.226768</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-11.559609</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-11.7438965</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-12.150990500000001</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-11.588990000000001</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'coordinates'!$C$2:$C$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>5.2652264000000004</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4.7514500000000002</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>5.0869289999999996</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8.0850609999999996</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>7.4355453999999996</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>9.2592649999999992</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>9.2371909999999993</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>9.7885030000000004</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8.5394410000000001</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>7.1614129999999996</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+              <c15:datalabelsRange>
+                <c15:f>'coordinates'!$A$2:$A$11</c15:f>
+                <c15:dlblRangeCache>
+                  <c:ptCount val="10"/>
                   <c:pt idx="0">
                     <c:v>v1</c:v>
                   </c:pt>
@@ -369,69 +863,231 @@
                   <c:pt idx="9">
                     <c:v>v10</c:v>
                   </c:pt>
-                </c:lvl>
-              </c:multiLvlStrCache>
-            </c:multiLvlStrRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>'coordinates'!$C$2:$C$11</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
+                </c15:dlblRangeCache>
+              </c15:datalabelsRange>
+            </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-F30F-4C7C-977D-7D7A46568CF0}"/>
+              <c16:uniqueId val="{00000002-F99D-46D1-A11D-727F70D9B603}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
         <c:dLbls>
+          <c:dLblPos val="t"/>
           <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
+          <c:showVal val="1"/>
           <c:showCatName val="0"/>
           <c:showSerName val="0"/>
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="722879183"/>
-        <c:axId val="722876783"/>
+        <c:axId val="1582521472"/>
+        <c:axId val="1582523872"/>
+        <c:extLst>
+          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+            <c15:filteredScatterSeries>
+              <c15:ser>
+                <c:idx val="0"/>
+                <c:order val="0"/>
+                <c:tx>
+                  <c:strRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'coordinates'!$C$1</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:strCache>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>y</c:v>
+                      </c:pt>
+                    </c:strCache>
+                  </c:strRef>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="38100" cap="rnd">
+                    <a:noFill/>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="circle"/>
+                  <c:size val="5"/>
+                  <c:spPr>
+                    <a:solidFill>
+                      <a:schemeClr val="accent1"/>
+                    </a:solidFill>
+                    <a:ln w="9525">
+                      <a:solidFill>
+                        <a:schemeClr val="accent1"/>
+                      </a:solidFill>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c:marker>
+                <c:dLbls>
+                  <c:spPr>
+                    <a:noFill/>
+                    <a:ln>
+                      <a:noFill/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                  <c:txPr>
+                    <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                      <a:spAutoFit/>
+                    </a:bodyPr>
+                    <a:lstStyle/>
+                    <a:p>
+                      <a:pPr>
+                        <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                          <a:solidFill>
+                            <a:schemeClr val="tx1">
+                              <a:lumMod val="75000"/>
+                              <a:lumOff val="25000"/>
+                            </a:schemeClr>
+                          </a:solidFill>
+                          <a:latin typeface="+mn-lt"/>
+                          <a:ea typeface="+mn-ea"/>
+                          <a:cs typeface="+mn-cs"/>
+                        </a:defRPr>
+                      </a:pPr>
+                      <a:endParaRPr lang="fr-FR"/>
+                    </a:p>
+                  </c:txPr>
+                  <c:dLblPos val="t"/>
+                  <c:showLegendKey val="0"/>
+                  <c:showVal val="1"/>
+                  <c:showCatName val="0"/>
+                  <c:showSerName val="0"/>
+                  <c:showPercent val="0"/>
+                  <c:showBubbleSize val="0"/>
+                  <c:showLeaderLines val="0"/>
+                  <c:extLst>
+                    <c:ext uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                      <c15:showLeaderLines val="1"/>
+                      <c15:leaderLines>
+                        <c:spPr>
+                          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                            <a:solidFill>
+                              <a:schemeClr val="tx1">
+                                <a:lumMod val="35000"/>
+                                <a:lumOff val="65000"/>
+                              </a:schemeClr>
+                            </a:solidFill>
+                            <a:round/>
+                          </a:ln>
+                          <a:effectLst/>
+                        </c:spPr>
+                      </c15:leaderLines>
+                    </c:ext>
+                  </c:extLst>
+                </c:dLbls>
+                <c:xVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'coordinates'!$B$2:$B$11</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="10"/>
+                      <c:pt idx="0">
+                        <c:v>-8.9920439999999999</c:v>
+                      </c:pt>
+                      <c:pt idx="1">
+                        <c:v>-8.9748190000000001</c:v>
+                      </c:pt>
+                      <c:pt idx="2">
+                        <c:v>-8.4463539999999995</c:v>
+                      </c:pt>
+                      <c:pt idx="3">
+                        <c:v>-11.709638</c:v>
+                      </c:pt>
+                      <c:pt idx="4">
+                        <c:v>-12.038005</c:v>
+                      </c:pt>
+                      <c:pt idx="5">
+                        <c:v>-12.226768</c:v>
+                      </c:pt>
+                      <c:pt idx="6">
+                        <c:v>-11.559609</c:v>
+                      </c:pt>
+                      <c:pt idx="7">
+                        <c:v>-11.7438965</c:v>
+                      </c:pt>
+                      <c:pt idx="8">
+                        <c:v>-12.150990500000001</c:v>
+                      </c:pt>
+                      <c:pt idx="9">
+                        <c:v>-11.588990000000001</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:xVal>
+                <c:yVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'coordinates'!$C$2:$C$11</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="10"/>
+                      <c:pt idx="0">
+                        <c:v>5.2652264000000004</c:v>
+                      </c:pt>
+                      <c:pt idx="1">
+                        <c:v>4.7514500000000002</c:v>
+                      </c:pt>
+                      <c:pt idx="2">
+                        <c:v>5.0869289999999996</c:v>
+                      </c:pt>
+                      <c:pt idx="3">
+                        <c:v>8.0850609999999996</c:v>
+                      </c:pt>
+                      <c:pt idx="4">
+                        <c:v>7.4355453999999996</c:v>
+                      </c:pt>
+                      <c:pt idx="5">
+                        <c:v>9.2592649999999992</c:v>
+                      </c:pt>
+                      <c:pt idx="6">
+                        <c:v>9.2371909999999993</c:v>
+                      </c:pt>
+                      <c:pt idx="7">
+                        <c:v>9.7885030000000004</c:v>
+                      </c:pt>
+                      <c:pt idx="8">
+                        <c:v>8.5394410000000001</c:v>
+                      </c:pt>
+                      <c:pt idx="9">
+                        <c:v>7.1614129999999996</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:yVal>
+                <c:smooth val="0"/>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000000-F99D-46D1-A11D-727F70D9B603}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredScatterSeries>
+          </c:ext>
+        </c:extLst>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="722879183"/>
+        <c:axId val="1582521472"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -451,7 +1107,8 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:majorTickMark val="none"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
@@ -487,12 +1144,12 @@
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="722876783"/>
+        <c:crossAx val="1582523872"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="722876783"/>
+        <c:axId val="1582523872"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -513,7 +1170,7 @@
           </c:spPr>
         </c:majorGridlines>
         <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
@@ -549,7 +1206,7 @@
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="722879183"/>
+        <c:crossAx val="1582521472"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -564,13 +1221,6 @@
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -606,6 +1256,671 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="fr-FR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'coordinates'!$C$38</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>y</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="38100" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="0"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{87546E47-BD2E-475E-82F9-6F049F246A1B}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[PLAGECELL]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="fr-FR"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000002-6BE9-4DE6-9CC6-00556339EE92}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{A78BDD45-4A27-4F56-AEAB-737BE3027936}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[PLAGECELL]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="fr-FR"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000003-6BE9-4DE6-9CC6-00556339EE92}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="2"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{3F5727E6-06F7-4935-AC84-308F614BE2EB}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[PLAGECELL]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="fr-FR"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000004-6BE9-4DE6-9CC6-00556339EE92}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="3"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{8D9634E4-8D44-4189-AEBC-822980E33472}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[PLAGECELL]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="fr-FR"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000005-6BE9-4DE6-9CC6-00556339EE92}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="4"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{53509D07-2EE6-4D80-A25E-901790CC3D14}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[PLAGECELL]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="fr-FR"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000006-6BE9-4DE6-9CC6-00556339EE92}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="5"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{39F50797-9857-4DAE-8031-D4FD490CD262}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[PLAGECELL]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="fr-FR"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000007-6BE9-4DE6-9CC6-00556339EE92}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="6"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{1395843B-C8F5-46E0-9D95-5544FFCF8EAE}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[PLAGECELL]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="fr-FR"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000008-6BE9-4DE6-9CC6-00556339EE92}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="7"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{9C15F6ED-FA10-4DB1-8EC7-6395CA06C5B9}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[PLAGECELL]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="fr-FR"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000009-6BE9-4DE6-9CC6-00556339EE92}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="8"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{63305337-0EFD-4270-80E0-42AB5D0E38FA}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[PLAGECELL]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="fr-FR"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{0000000A-6BE9-4DE6-9CC6-00556339EE92}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="9"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:fld id="{609004DE-B21A-4CDC-9848-F5EEEFB618E2}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[PLAGECELL]</a:t>
+                    </a:fld>
+                    <a:endParaRPr lang="fr-FR"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
+                  <c15:showDataLabelsRange val="1"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{0000000B-6BE9-4DE6-9CC6-00556339EE92}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="fr-FR"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="t"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showDataLabelsRange val="1"/>
+                <c15:showLeaderLines val="0"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'coordinates'!$B$39:$B$48</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>1.363156</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.1465540000000001</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.7815300000000001</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.0134980000000002</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2.6400790000000001</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2.3743420000000004</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3.2203459999999993</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.83608199999999933</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2.7240090000000006</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>3.2296929999999993</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'coordinates'!$C$39:$C$48</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>1.3474950000000003</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.75485600000000019</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.40410900000000005</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-4.0653999999999968E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.40200999999999976</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.8549490000000004</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.33934</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.088279</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.4697880000000003</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.59523499999999974</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+              <c15:datalabelsRange>
+                <c15:f>'coordinates'!$A$39:$A$48</c15:f>
+                <c15:dlblRangeCache>
+                  <c:ptCount val="10"/>
+                  <c:pt idx="0">
+                    <c:v>v1</c:v>
+                  </c:pt>
+                  <c:pt idx="1">
+                    <c:v>v2</c:v>
+                  </c:pt>
+                  <c:pt idx="2">
+                    <c:v>v3</c:v>
+                  </c:pt>
+                  <c:pt idx="3">
+                    <c:v>v4</c:v>
+                  </c:pt>
+                  <c:pt idx="4">
+                    <c:v>v5</c:v>
+                  </c:pt>
+                  <c:pt idx="5">
+                    <c:v>v6</c:v>
+                  </c:pt>
+                  <c:pt idx="6">
+                    <c:v>v7</c:v>
+                  </c:pt>
+                  <c:pt idx="7">
+                    <c:v>v8</c:v>
+                  </c:pt>
+                  <c:pt idx="8">
+                    <c:v>v9</c:v>
+                  </c:pt>
+                  <c:pt idx="9">
+                    <c:v>v10</c:v>
+                  </c:pt>
+                </c15:dlblRangeCache>
+              </c15:datalabelsRange>
+            </c:ext>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-6BE9-4DE6-9CC6-00556339EE92}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:dLblPos val="t"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1582521472"/>
+        <c:axId val="1439403216"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1582521472"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="1439403216"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1439403216"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="1582521472"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="fr-FR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="fr-FR"/>
@@ -941,7 +2256,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="fr-FR"/>
@@ -1387,6 +2702,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -2935,27 +4290,543 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>106680</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>41910</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>144780</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>716280</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>41910</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>502920</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="6" name="Graphique 5">
+        <xdr:cNvPr id="9" name="Graphique 8">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D4C8A99E-406E-B03A-91D2-22299F0BB5F4}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{47C1F8A5-8A83-D9A3-0749-A5343998524B}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2968,6 +4839,42 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>106680</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>11430</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>716280</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>11430</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="11" name="Graphique 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4C664BBE-6D69-C3FE-861E-CBA0D14820AE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3069,11 +4976,39 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4A2B3991-9238-4962-A830-2F8B446E49DB}" name="coordinates" displayName="coordinates" ref="A1:C11" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:C11" xr:uid="{4A2B3991-9238-4962-A830-2F8B446E49DB}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{B0F6DDC3-FCA2-4343-A812-5C577727C61A}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{DAAC643B-1FC2-4F00-AECB-4B39EE07D142}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{99058399-71C0-4F83-824B-673588F48D99}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{B0F6DDC3-FCA2-4343-A812-5C577727C61A}" uniqueName="1" name="label" queryTableFieldId="1" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{DAAC643B-1FC2-4F00-AECB-4B39EE07D142}" uniqueName="2" name="x" queryTableFieldId="2" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{99058399-71C0-4F83-824B-673588F48D99}" uniqueName="3" name="y" queryTableFieldId="3" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{76FCCB60-3154-45F8-9C01-E8FBD8AD8C35}" name="Tableau2" displayName="Tableau2" ref="A26:C36" totalsRowShown="0">
+  <autoFilter ref="A26:C36" xr:uid="{76FCCB60-3154-45F8-9C01-E8FBD8AD8C35}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{C961DDCD-3869-4616-BCCA-170379B9D59A}" name="l"/>
+    <tableColumn id="2" xr3:uid="{E5E79DBE-AD5B-436D-A999-991424DB644F}" name="x"/>
+    <tableColumn id="3" xr3:uid="{6781C77C-6365-4B94-A77C-33D0E702763E}" name="y"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{09D43346-4BC0-407A-AF9B-91EC74059A75}" name="Tableau3" displayName="Tableau3" ref="A38:C48" totalsRowShown="0">
+  <autoFilter ref="A38:C48" xr:uid="{09D43346-4BC0-407A-AF9B-91EC74059A75}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{74885210-6C4C-462C-8CD8-DEE30882CE1B}" name="l" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{347D7809-A8BA-442D-B8BC-021D85359900}" name="x">
+      <calculatedColumnFormula>B27-9</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="3" xr3:uid="{CAD4FF5F-3F0B-4966-9D0A-EBEC93CF7A9E}" name="y">
+      <calculatedColumnFormula>C27-5</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -3394,7 +5329,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{195DE73C-B8E2-4E3C-908B-055D77AB59B0}">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:D48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.6640625" bestFit="1" customWidth="1"/>
@@ -3402,132 +5337,401 @@
     <col min="3" max="3" width="10.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" t="s">
         <v>30</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>31</v>
       </c>
-      <c r="C1" t="s">
-        <v>32</v>
-      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>2</v>
+      <c r="B2">
+        <v>-8.9920439999999999</v>
+      </c>
+      <c r="C2">
+        <v>5.2652264000000004</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>5</v>
+      <c r="B3">
+        <v>-8.9748190000000001</v>
+      </c>
+      <c r="C3">
+        <v>4.7514500000000002</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>8</v>
+      <c r="B4">
+        <v>-8.4463539999999995</v>
+      </c>
+      <c r="C4">
+        <v>5.0869289999999996</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>11</v>
+      <c r="B5">
+        <v>-11.709638</v>
+      </c>
+      <c r="C5">
+        <v>8.0850609999999996</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>14</v>
+      <c r="B6">
+        <v>-12.038005</v>
+      </c>
+      <c r="C6">
+        <v>7.4355453999999996</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>17</v>
+      <c r="B7">
+        <v>-12.226768</v>
+      </c>
+      <c r="C7">
+        <v>9.2592649999999992</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>20</v>
+      <c r="B8">
+        <v>-11.559609</v>
+      </c>
+      <c r="C8">
+        <v>9.2371909999999993</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>23</v>
+      <c r="B9">
+        <v>-11.7438965</v>
+      </c>
+      <c r="C9">
+        <v>9.7885030000000004</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>26</v>
+      <c r="B10">
+        <v>-12.150990500000001</v>
+      </c>
+      <c r="C10">
+        <v>8.5394410000000001</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
         <v>27</v>
       </c>
-      <c r="B11" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>29</v>
+      <c r="B11">
+        <v>-11.588990000000001</v>
+      </c>
+      <c r="C11">
+        <v>7.1614129999999996</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D14">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>33</v>
+      </c>
+      <c r="B26" t="s">
+        <v>30</v>
+      </c>
+      <c r="C26" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>0</v>
+      </c>
+      <c r="B27">
+        <v>10.363156</v>
+      </c>
+      <c r="C27">
+        <v>6.3474950000000003</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>3</v>
+      </c>
+      <c r="B28">
+        <v>10.146554</v>
+      </c>
+      <c r="C28">
+        <v>5.7548560000000002</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>6</v>
+      </c>
+      <c r="B29">
+        <v>10.78153</v>
+      </c>
+      <c r="C29">
+        <v>5.4041090000000001</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>9</v>
+      </c>
+      <c r="B30">
+        <v>11.013498</v>
+      </c>
+      <c r="C30">
+        <v>4.959346</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>12</v>
+      </c>
+      <c r="B31">
+        <v>11.640079</v>
+      </c>
+      <c r="C31">
+        <v>5.4020099999999998</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>15</v>
+      </c>
+      <c r="B32">
+        <v>11.374342</v>
+      </c>
+      <c r="C32">
+        <v>6.8549490000000004</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>18</v>
+      </c>
+      <c r="B33">
+        <v>12.220345999999999</v>
+      </c>
+      <c r="C33">
+        <v>6.33934</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>21</v>
+      </c>
+      <c r="B34">
+        <v>9.8360819999999993</v>
+      </c>
+      <c r="C34">
+        <v>6.088279</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>24</v>
+      </c>
+      <c r="B35">
+        <v>11.724009000000001</v>
+      </c>
+      <c r="C35">
+        <v>6.4697880000000003</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>27</v>
+      </c>
+      <c r="B36">
+        <v>12.229692999999999</v>
+      </c>
+      <c r="C36">
+        <v>5.5952349999999997</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>33</v>
+      </c>
+      <c r="B38" t="s">
+        <v>30</v>
+      </c>
+      <c r="C38" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B39">
+        <f>B27-9</f>
+        <v>1.363156</v>
+      </c>
+      <c r="C39">
+        <f>C27-5</f>
+        <v>1.3474950000000003</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B40">
+        <f t="shared" ref="B40:B48" si="0">B28-9</f>
+        <v>1.1465540000000001</v>
+      </c>
+      <c r="C40">
+        <f t="shared" ref="C40:C48" si="1">C28-5</f>
+        <v>0.75485600000000019</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B41">
+        <f t="shared" si="0"/>
+        <v>1.7815300000000001</v>
+      </c>
+      <c r="C41">
+        <f t="shared" si="1"/>
+        <v>0.40410900000000005</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B42">
+        <f t="shared" si="0"/>
+        <v>2.0134980000000002</v>
+      </c>
+      <c r="C42">
+        <f t="shared" si="1"/>
+        <v>-4.0653999999999968E-2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B43">
+        <f t="shared" si="0"/>
+        <v>2.6400790000000001</v>
+      </c>
+      <c r="C43">
+        <f t="shared" si="1"/>
+        <v>0.40200999999999976</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A44" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B44">
+        <f t="shared" si="0"/>
+        <v>2.3743420000000004</v>
+      </c>
+      <c r="C44">
+        <f t="shared" si="1"/>
+        <v>1.8549490000000004</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A45" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B45">
+        <f t="shared" si="0"/>
+        <v>3.2203459999999993</v>
+      </c>
+      <c r="C45">
+        <f t="shared" si="1"/>
+        <v>1.33934</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A46" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B46">
+        <f t="shared" si="0"/>
+        <v>0.83608199999999933</v>
+      </c>
+      <c r="C46">
+        <f t="shared" si="1"/>
+        <v>1.088279</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A47" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B47">
+        <f t="shared" si="0"/>
+        <v>2.7240090000000006</v>
+      </c>
+      <c r="C47">
+        <f t="shared" si="1"/>
+        <v>1.4697880000000003</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A48" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B48">
+        <f t="shared" si="0"/>
+        <v>3.2296929999999993</v>
+      </c>
+      <c r="C48">
+        <f t="shared" si="1"/>
+        <v>0.59523499999999974</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
-  <tableParts count="1">
+  <tableParts count="3">
     <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>